<commit_message>
publish: 5f71a562033199c430276eda7f30b64f39010936 (run 30470599429)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.1.0</t>
+    <t>0.2.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-07-29T14:03:51+00:00</t>
+    <t>2026-07-29T16:26:07+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: f956dfbf9adf3f753614ee2bdec533ef5e53615f (run 31026905231)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.0</t>
+    <t>0.2.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-05T16:28:11+00:00</t>
+    <t>2026-08-05T16:48:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 903b7ee739be56e282cd8ca89d6cbb8125e4b352 (run 31989785705)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.1</t>
+    <t>0.2.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-05T16:48:01+00:00</t>
+    <t>2026-08-17T03:02:16+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 6eddc4d72a9e3845de2de47a98298f41750a4da5 (run 31997886440)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.3</t>
+    <t>0.2.4</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-17T03:02:16+00:00</t>
+    <t>2026-08-17T05:27:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 85f79b2cbc79dea76cd233ba159d0916e90e8c0d (run 32003633416)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.4</t>
+    <t>0.2.5</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-17T05:27:05+00:00</t>
+    <t>2026-08-17T06:57:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 70ba822b088d4b9cbb72ff223e46c5851a15f4fb (run 32366652194)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.2.5</t>
+    <t>0.3.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-17T06:57:01+00:00</t>
+    <t>2026-08-20T12:04:33+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 0a869d80bbb070d36071f6529fdc9bc10e66a786 (run 32375379493)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.3.3</t>
+    <t>0.4.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T12:04:33+00:00</t>
+    <t>2026-08-20T13:40:11+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 19b16f8eff353acb13aa885d7e3068e28d03ccb1 (run 32392658430)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.4.0</t>
+    <t>0.5.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T13:40:11+00:00</t>
+    <t>2026-08-20T16:35:38+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 300be95f97739d291fd9b1f41f4dfe008284987d (run 32398610786)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.5.0</t>
+    <t>0.6.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T16:35:38+00:00</t>
+    <t>2026-08-20T17:39:23+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 3761368983d21858d659f16c83991defa3d6c52c (run 32401836568)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.0</t>
+    <t>0.6.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T17:39:23+00:00</t>
+    <t>2026-08-20T18:13:29+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 77f49b0a1c648c9eb5d6d31c9f39c7c051cbb026 (run 32431846411)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.1</t>
+    <t>0.6.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-20T18:13:29+00:00</t>
+    <t>2026-08-21T00:14:56+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 46a29fc5e272a6c2c412d4709cdf7733dee63006 (run 32434643455)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.6.2</t>
+    <t>0.7.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -48,7 +48,7 @@
     <t>Status</t>
   </si>
   <si>
-    <t>active</t>
+    <t>draft</t>
   </si>
   <si>
     <t>Experimental</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T00:14:56+00:00</t>
+    <t>2026-08-21T00:59:40+00:00</t>
   </si>
   <si>
     <t>Publisher</t>
@@ -87,7 +87,7 @@
     <t>Description</t>
   </si>
   <si>
-    <t>將 CS-Appendix10Operation（附表十 35 項具名作業）對映至 CS-HazardType（12 危害家族）。每一具名作業（source）相對於其對應之危害家族（target）在語意上較窄，故 equivalence = narrower（家族涵蓋範圍較廣）。供接收端由法定作業編號歸併至危害家族，回應審查意見之逐號可追溯性需求。</t>
+    <t>【依據：勞工健康保護規則附表】將 CS-Appendix10Operation（附表十 35 項具名作業）對映至 CS-HazardType（12 危害家族）。每一具名作業（source）相對於其對應之危害家族（target）在語意上較窄，故 equivalence = narrower（家族涵蓋範圍較廣）。供接收端由法定作業編號歸併至危害家族，回應審查意見之逐號可追溯性需求。</t>
   </si>
   <si>
     <t>Purpose</t>

</xml_diff>

<commit_message>
publish: f09302dc1af7bdb4091f974e02ecd5b087e82e45 (run 32436025618)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.7.0</t>
+    <t>0.7.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T00:59:40+00:00</t>
+    <t>2026-08-21T01:22:55+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 336a0b9c5ed19606bc98c8433375fbcefd01a7a2 (run 32446541457)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.7.1</t>
+    <t>0.8.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T01:22:55+00:00</t>
+    <t>2026-08-21T04:20:36+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 4f7021df32df91c62a7a9b3ac67fbda9b4595ff2 (run 32482292165)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.8.1</t>
+    <t>0.8.5</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T04:20:36+00:00</t>
+    <t>2026-08-21T12:32:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 6371a1de6267030716eac8d65787db2346d53ff1 (run 32492141395)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.8.5</t>
+    <t>0.9.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T12:32:47+00:00</t>
+    <t>2026-08-21T14:27:31+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 114c312a7aed3b3562677a074dd609d279898270 (run 32495634441)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.0</t>
+    <t>0.9.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T14:27:31+00:00</t>
+    <t>2026-08-21T15:06:05+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 39a3dcc7d98eccdf9dc64627b776be19f205d8f4 (run 32501027453)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.2</t>
+    <t>0.9.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T15:06:05+00:00</t>
+    <t>2026-08-21T16:05:47+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 65e1a8516e81ac13aba5f7daabe5c3b1f789449e (run 32545631906)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.9.3</t>
+    <t>0.10.0</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-21T16:05:47+00:00</t>
+    <t>2026-08-22T02:14:01+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 557e36b82036ed7a38cb8fa1034bf144444642aa (run 32562490363)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.10.0</t>
+    <t>0.10.1</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-22T04:25:10+00:00</t>
+    <t>2026-08-22T08:31:54+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 29053f19ffd2318fc1cd402c8d92aff148f9df27 (run 32577620247)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.10.1</t>
+    <t>0.10.2</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-22T08:31:54+00:00</t>
+    <t>2026-08-22T14:05:28+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>

<commit_message>
publish: 8223e3ccdf3e4c4cfb4c0fe9b758dc228622397d (run 32586773893)
</commit_message>
<xml_diff>
--- a/Appendix10-to-HazardType.xlsx
+++ b/Appendix10-to-HazardType.xlsx
@@ -30,7 +30,7 @@
     <t>Version</t>
   </si>
   <si>
-    <t>0.10.2</t>
+    <t>0.10.3</t>
   </si>
   <si>
     <t>Name</t>
@@ -60,7 +60,7 @@
     <t>Date</t>
   </si>
   <si>
-    <t>2026-08-22T14:05:28+00:00</t>
+    <t>2026-08-22T17:09:34+00:00</t>
   </si>
   <si>
     <t>Publisher</t>

</xml_diff>